<commit_message>
chore: update GitHub Repos export
</commit_message>
<xml_diff>
--- a/dist/repos.xlsx
+++ b/dist/repos.xlsx
@@ -606,7 +606,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>github-repos</t>
+          <t>github-repos，https://abc1319.github.io/github-repos/</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr"/>
@@ -639,12 +639,12 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05T05:17:18Z</t>
+          <t>2026-08-05T05:23:50Z</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05T05:17:17Z</t>
+          <t>2026-08-05T05:21:33Z</t>
         </is>
       </c>
       <c r="P2" s="2" t="n">

</xml_diff>